<commit_message>
NPB自動更新(2軍): 2026-09-19 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/2軍/公式戦/raw/2026-09-19/highlights_20260919.xlsx
+++ b/data/プロ野球/2026年/2軍/公式戦/raw/2026-09-19/highlights_20260919.xlsx
@@ -454,17 +454,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>皆川 岳飛</t>
+          <t>若林 楽人</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>巨人</t>
+          <t>西武</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>7回裏に逆転2ランホームランを放ち、試合の主導権を奪い返す劇的な一打となった。</t>
+          <t>1回表に先制弾、3回表には同点弾を放ち、2本塁打でチームを牽引した。</t>
         </is>
       </c>
     </row>
@@ -479,17 +479,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>中山 翔太</t>
+          <t>皆川 岳飛</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>オイシックス</t>
+          <t>巨人</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>9回表に決勝ホームランを放ち、チームを勝利に導く劇的な活躍を見せた。</t>
+          <t>7回裏にライトスタンドへ逆転2ランを放ち、試合の流れを大きく引き寄せた。</t>
         </is>
       </c>
     </row>
@@ -504,17 +504,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>若林 楽人</t>
+          <t>中山 翔太</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>西武</t>
+          <t>オイシックス</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1試合2本塁打の活躍。先制弾と3回裏の同点弾で打線を牽引した。</t>
+          <t>9回表に決勝となるソロホームランを放ち、チームを勝利に導いた。</t>
         </is>
       </c>
     </row>
@@ -529,17 +529,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>山村 崇嘉</t>
+          <t>横山 聖哉</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>西武</t>
+          <t>オリックス</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9回表に同点犠牲フライを放ち、土壇場でチームの窮地を救う活躍を見せた。</t>
+          <t>9回表に満塁のチャンスで勝ち越しタイムリーを放ち、チームの勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -554,17 +554,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>横山 聖哉</t>
+          <t>ラミレス</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>オリックス</t>
+          <t>広島</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>9回表に勝ち越しタイムリーヒットを放ち、接戦を制する貴重な一打となった。</t>
+          <t>8回裏に同点となるタイムリーツーベースを放ち、試合を振り出しに戻した。</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ラミレス</t>
+          <t>矢澤 宏太</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>広島</t>
+          <t>日本ハム</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8回裏に同点タイムリーツーベースを放ち、土壇場で試合を振り出しに戻した。</t>
+          <t>9回表にダメ押しとなる2ランホームランを放ち、チームの勝利を決定づけた。</t>
         </is>
       </c>
     </row>

</xml_diff>